<commit_message>
Add eta_sub, EQE and spectral-average checks to series vs eq. (3) raw data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpyv6uQaiqNNFK2eUPJ4BU
</commit_message>
<xml_diff>
--- a/figures/fig2e_series_vs_eq3/fig2e_series_vs_eq3_rawdata.xlsx
+++ b/figures/fig2e_series_vs_eq3/fig2e_series_vs_eq3_rawdata.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="c_eta_ext" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="d_difference" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cutoffs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQE_check" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spectral_avg_check" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="d_difference" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cutoffs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,7 +474,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sheet c: panel (c), solid = series, dashed = eq. (3).  Sheet d: panel (d), difference series - eq. (3) in percentage points.</t>
+          <t>Sheet c: panel (c), solid = series, dashed = eq. (3), thin = eta_sub. Sheet EQE_check: EQE = eta_sub x eta_ext rises monotonically (no dips).  Sheet d: panel (d), difference series - eq. (3) in percentage points.</t>
         </is>
       </c>
     </row>
@@ -501,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -519,22 +521,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Al series</t>
+          <t>Al eta_ext series</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Al eq. (3)</t>
+          <t>Al eta_ext eq. (3)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ag series</t>
+          <t>Ag eta_ext series</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Ag eq. (3)</t>
+          <t>Ag eta_ext eq. (3)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Al eta_sub</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ag eta_sub</t>
         </is>
       </c>
     </row>
@@ -554,6 +566,12 @@
       <c r="E2" t="n">
         <v>0.982445</v>
       </c>
+      <c r="F2" t="n">
+        <v>0.264561</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.313559</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -571,6 +589,12 @@
       <c r="E3" t="n">
         <v>0.981858</v>
       </c>
+      <c r="F3" t="n">
+        <v>0.268021</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.316572</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -588,6 +612,12 @@
       <c r="E4" t="n">
         <v>0.9813</v>
       </c>
+      <c r="F4" t="n">
+        <v>0.271705</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.319724</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -605,6 +635,12 @@
       <c r="E5" t="n">
         <v>0.980696</v>
       </c>
+      <c r="F5" t="n">
+        <v>0.275651</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.323038</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -622,6 +658,12 @@
       <c r="E6" t="n">
         <v>0.9800450000000001</v>
       </c>
+      <c r="F6" t="n">
+        <v>0.279908</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.326538</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -639,6 +681,12 @@
       <c r="E7" t="n">
         <v>0.979414</v>
       </c>
+      <c r="F7" t="n">
+        <v>0.284534</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.330255</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -656,6 +704,12 @@
       <c r="E8" t="n">
         <v>0.978762</v>
       </c>
+      <c r="F8" t="n">
+        <v>0.289606</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.334229</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -673,6 +727,12 @@
       <c r="E9" t="n">
         <v>0.978154</v>
       </c>
+      <c r="F9" t="n">
+        <v>0.295219</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.338505</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -690,6 +750,12 @@
       <c r="E10" t="n">
         <v>0.977453</v>
       </c>
+      <c r="F10" t="n">
+        <v>0.301494</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.343144</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -707,6 +773,12 @@
       <c r="E11" t="n">
         <v>0.976733</v>
       </c>
+      <c r="F11" t="n">
+        <v>0.308592</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.34822</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -724,6 +796,12 @@
       <c r="E12" t="n">
         <v>0.975961</v>
       </c>
+      <c r="F12" t="n">
+        <v>0.316716</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.353833</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -741,6 +819,12 @@
       <c r="E13" t="n">
         <v>0.975162</v>
       </c>
+      <c r="F13" t="n">
+        <v>0.326116</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.360115</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -758,6 +842,12 @@
       <c r="E14" t="n">
         <v>0.974369</v>
       </c>
+      <c r="F14" t="n">
+        <v>0.33704</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.367244</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -775,6 +865,12 @@
       <c r="E15" t="n">
         <v>0.973202</v>
       </c>
+      <c r="F15" t="n">
+        <v>0.349471</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.375474</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -792,6 +888,12 @@
       <c r="E16" t="n">
         <v>0.972411</v>
       </c>
+      <c r="F16" t="n">
+        <v>0.362068</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.385169</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -809,6 +911,12 @@
       <c r="E17" t="n">
         <v>0.971162</v>
       </c>
+      <c r="F17" t="n">
+        <v>0.371693</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.396883</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -826,6 +934,12 @@
       <c r="E18" t="n">
         <v>0.969915</v>
       </c>
+      <c r="F18" t="n">
+        <v>0.378342</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.411491</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -843,6 +957,12 @@
       <c r="E19" t="n">
         <v>0.968359</v>
       </c>
+      <c r="F19" t="n">
+        <v>0.383587</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.430406</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -860,6 +980,12 @@
       <c r="E20" t="n">
         <v>0.966154</v>
       </c>
+      <c r="F20" t="n">
+        <v>0.388214</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.45509</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -877,6 +1003,12 @@
       <c r="E21" t="n">
         <v>0.9651459999999999</v>
       </c>
+      <c r="F21" t="n">
+        <v>0.392602</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.469168</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -894,6 +1026,12 @@
       <c r="E22" t="n">
         <v>0.964401</v>
       </c>
+      <c r="F22" t="n">
+        <v>0.396981</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.474062</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -911,6 +1049,12 @@
       <c r="E23" t="n">
         <v>0.963734</v>
       </c>
+      <c r="F23" t="n">
+        <v>0.401527</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.478258</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -928,6 +1072,12 @@
       <c r="E24" t="n">
         <v>0.963152</v>
       </c>
+      <c r="F24" t="n">
+        <v>0.406411</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.482489</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -945,6 +1095,12 @@
       <c r="E25" t="n">
         <v>0.962426</v>
       </c>
+      <c r="F25" t="n">
+        <v>0.411836</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.487036</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -962,6 +1118,12 @@
       <c r="E26" t="n">
         <v>0.9617019999999999</v>
       </c>
+      <c r="F26" t="n">
+        <v>0.418078</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.492132</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -979,6 +1141,12 @@
       <c r="E27" t="n">
         <v>0.960934</v>
       </c>
+      <c r="F27" t="n">
+        <v>0.425557</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.498066</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -996,6 +1164,12 @@
       <c r="E28" t="n">
         <v>0.960057</v>
       </c>
+      <c r="F28" t="n">
+        <v>0.434975</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.505283</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1013,6 +1187,12 @@
       <c r="E29" t="n">
         <v>0.959103</v>
       </c>
+      <c r="F29" t="n">
+        <v>0.447634</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.514551</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1030,6 +1210,12 @@
       <c r="E30" t="n">
         <v>0.95797</v>
       </c>
+      <c r="F30" t="n">
+        <v>0.46627</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.5273870000000001</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1047,6 +1233,12 @@
       <c r="E31" t="n">
         <v>0.956396</v>
       </c>
+      <c r="F31" t="n">
+        <v>0.497473</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.547331</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1064,6 +1256,12 @@
       <c r="E32" t="n">
         <v>0.953958</v>
       </c>
+      <c r="F32" t="n">
+        <v>0.542357</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.58497</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1081,6 +1279,12 @@
       <c r="E33" t="n">
         <v>0.951751</v>
       </c>
+      <c r="F33" t="n">
+        <v>0.559001</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.6288820000000001</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1098,6 +1302,12 @@
       <c r="E34" t="n">
         <v>0.951128</v>
       </c>
+      <c r="F34" t="n">
+        <v>0.569117</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.638906</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1115,6 +1325,12 @@
       <c r="E35" t="n">
         <v>0.949978</v>
       </c>
+      <c r="F35" t="n">
+        <v>0.577955</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.647304</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1132,6 +1348,12 @@
       <c r="E36" t="n">
         <v>0.950035</v>
       </c>
+      <c r="F36" t="n">
+        <v>0.586514</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.655663</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1149,6 +1371,12 @@
       <c r="E37" t="n">
         <v>0.949512</v>
       </c>
+      <c r="F37" t="n">
+        <v>0.59518</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.664357</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1166,6 +1394,12 @@
       <c r="E38" t="n">
         <v>0.948997</v>
       </c>
+      <c r="F38" t="n">
+        <v>0.60417</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.673574</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1183,6 +1417,12 @@
       <c r="E39" t="n">
         <v>0.948478</v>
       </c>
+      <c r="F39" t="n">
+        <v>0.613644</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.683466</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1200,6 +1440,12 @@
       <c r="E40" t="n">
         <v>0.948034</v>
       </c>
+      <c r="F40" t="n">
+        <v>0.623746</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.69418</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1217,6 +1463,12 @@
       <c r="E41" t="n">
         <v>0.947488</v>
       </c>
+      <c r="F41" t="n">
+        <v>0.634624</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.705883</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1234,6 +1486,12 @@
       <c r="E42" t="n">
         <v>0.946612</v>
       </c>
+      <c r="F42" t="n">
+        <v>0.646443</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.718771</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1251,6 +1509,12 @@
       <c r="E43" t="n">
         <v>0.946232</v>
       </c>
+      <c r="F43" t="n">
+        <v>0.659395</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.733088</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1268,6 +1532,12 @@
       <c r="E44" t="n">
         <v>0.945576</v>
       </c>
+      <c r="F44" t="n">
+        <v>0.67371</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.749139</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1285,6 +1555,12 @@
       <c r="E45" t="n">
         <v>0.94474</v>
       </c>
+      <c r="F45" t="n">
+        <v>0.689666</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.7673219999999999</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1302,6 +1578,12 @@
       <c r="E46" t="n">
         <v>0.943361</v>
       </c>
+      <c r="F46" t="n">
+        <v>0.707593</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.788151</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1319,6 +1601,12 @@
       <c r="E47" t="n">
         <v>0.942232</v>
       </c>
+      <c r="F47" t="n">
+        <v>0.72784</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.812313</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1336,6 +1624,12 @@
       <c r="E48" t="n">
         <v>0.940437</v>
       </c>
+      <c r="F48" t="n">
+        <v>0.750566</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.840706</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1353,6 +1647,12 @@
       <c r="E49" t="n">
         <v>0.937747</v>
       </c>
+      <c r="F49" t="n">
+        <v>0.774911</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.874421</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1370,6 +1670,12 @@
       <c r="E50" t="n">
         <v>0.933805</v>
       </c>
+      <c r="F50" t="n">
+        <v>0.801322</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.912875</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1387,6 +1693,12 @@
       <c r="E51" t="n">
         <v>0.930661</v>
       </c>
+      <c r="F51" t="n">
+        <v>0.831473</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.94474</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1404,6 +1716,12 @@
       <c r="E52" t="n">
         <v>0.929019</v>
       </c>
+      <c r="F52" t="n">
+        <v>0.8414779999999999</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.956185</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1421,6 +1739,12 @@
       <c r="E53" t="n">
         <v>0.928399</v>
       </c>
+      <c r="F53" t="n">
+        <v>0.842928</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.95756</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1438,6 +1762,12 @@
       <c r="E54" t="n">
         <v>0.9278189999999999</v>
       </c>
+      <c r="F54" t="n">
+        <v>0.84367</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.958201</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1455,6 +1785,12 @@
       <c r="E55" t="n">
         <v>0.926256</v>
       </c>
+      <c r="F55" t="n">
+        <v>0.844252</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.958649</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1472,6 +1808,12 @@
       <c r="E56" t="n">
         <v>0.9266529999999999</v>
       </c>
+      <c r="F56" t="n">
+        <v>0.844799</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.958959</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1489,6 +1831,12 @@
       <c r="E57" t="n">
         <v>0.926107</v>
       </c>
+      <c r="F57" t="n">
+        <v>0.845467</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.959183</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1506,6 +1854,12 @@
       <c r="E58" t="n">
         <v>0.925623</v>
       </c>
+      <c r="F58" t="n">
+        <v>0.846455</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.959363</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1523,6 +1877,12 @@
       <c r="E59" t="n">
         <v>0.9250969999999999</v>
       </c>
+      <c r="F59" t="n">
+        <v>0.8478599999999999</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.959554</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1540,6 +1900,12 @@
       <c r="E60" t="n">
         <v>0.924226</v>
       </c>
+      <c r="F60" t="n">
+        <v>0.849248</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.959637</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1557,6 +1923,12 @@
       <c r="E61" t="n">
         <v>0.924038</v>
       </c>
+      <c r="F61" t="n">
+        <v>0.850395</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.9597599999999999</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1574,6 +1946,12 @@
       <c r="E62" t="n">
         <v>0.923517</v>
       </c>
+      <c r="F62" t="n">
+        <v>0.851217</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.9598640000000001</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1591,6 +1969,12 @@
       <c r="E63" t="n">
         <v>0.923059</v>
       </c>
+      <c r="F63" t="n">
+        <v>0.851797</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.959961</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1608,6 +1992,12 @@
       <c r="E64" t="n">
         <v>0.922566</v>
       </c>
+      <c r="F64" t="n">
+        <v>0.852176</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.960012</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1625,6 +2015,12 @@
       <c r="E65" t="n">
         <v>0.921346</v>
       </c>
+      <c r="F65" t="n">
+        <v>0.852476</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.960109</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1642,6 +2038,12 @@
       <c r="E66" t="n">
         <v>0.921535</v>
       </c>
+      <c r="F66" t="n">
+        <v>0.852665</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.960166</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1659,6 +2061,12 @@
       <c r="E67" t="n">
         <v>0.9210429999999999</v>
       </c>
+      <c r="F67" t="n">
+        <v>0.8527979999999999</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.960224</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1676,6 +2084,12 @@
       <c r="E68" t="n">
         <v>0.9205950000000001</v>
       </c>
+      <c r="F68" t="n">
+        <v>0.852876</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.960266</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1693,6 +2107,12 @@
       <c r="E69" t="n">
         <v>0.920126</v>
       </c>
+      <c r="F69" t="n">
+        <v>0.852947</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.960337</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1710,6 +2130,12 @@
       <c r="E70" t="n">
         <v>0.919403</v>
       </c>
+      <c r="F70" t="n">
+        <v>0.852962</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0.960364</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1727,6 +2153,12 @@
       <c r="E71" t="n">
         <v>0.919029</v>
       </c>
+      <c r="F71" t="n">
+        <v>0.8529640000000001</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.9603969999999999</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1743,6 +2175,12 @@
       </c>
       <c r="E72" t="n">
         <v>0.9185990000000001</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.852951</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0.960427</v>
       </c>
     </row>
   </sheetData>
@@ -1751,6 +2189,2506 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G72"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>n_sub (= n_MLA)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Al EQE series</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Al EQE eq. (3)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Ag EQE series</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ag EQE eq. (3)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Al dEQE_series/dn step</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ag dEQE_series/dn step</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.242404</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.242126</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.307735</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.308055</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.244806</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.244519</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.310669</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.310829</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.00293</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.24726</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.247062</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.313707</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.313745</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.00245</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.00304</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.249783</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.249783</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.316854</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.316802</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.00252</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.00315</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.252388</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.252716</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.320135</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.320022</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.00328</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.255092</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.255903</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.323594</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.323457</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.00346</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.258015</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.259501</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.327265</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.32713</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.00292</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.00367</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.261075</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.263485</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.331193</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.33111</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.00306</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.00393</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.264283</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.267943</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.335394</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.335407</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.00321</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0042</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.267646</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.272989</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.339942</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.340118</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.00336</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.00455</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.271161</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.278767</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.344902</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.345327</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.00351</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.00496</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.274937</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.285567</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.350379</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.35117</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.00378</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.00548</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.278843</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.29345</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.356486</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.357832</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.00391</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.00611</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.282836</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.302371</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.36326</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.365412</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.00399</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.00677</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.286854</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.311277</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.371074</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.374542</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.00402</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.00781</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.290872</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.317819</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.37988</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.385438</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.00402</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.00881</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.29496</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.322184</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.389983</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.399112</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.00409</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0101</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.298962</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.325454</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.401205</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.416788</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.01122</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.30287</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.328226</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.41249</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.439687</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.00391</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.01129</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.306688</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.330786</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.42329</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.452815</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.00382</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0108</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.310433</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.333306</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.431991</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.457185</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.00374</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.008699999999999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.314305</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.336062</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.439335</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.460914</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.00387</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.00734</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.318199</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.339045</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.44587</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.464711</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.00389</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.00654</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.322183</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.342407</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.451941</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.468736</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.00398</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.00607</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.326354</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.346355</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.457946</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.473284</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.00417</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.00601</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.330849</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.351207</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.464183</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.478609</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.0045</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.00624</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0.336054</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.357633</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.471059</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.4851</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.00521</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.00688</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.342103</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.366497</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.479055</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.493507</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.00605</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.008</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.349415</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.379886</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.488981</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.505221</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.00731</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.00993</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="B31" t="n">
+        <v>0.358374</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.402811</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.502183</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.523465</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.008959999999999999</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.0132</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="B32" t="n">
+        <v>0.368625</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.435993</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.520448</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.558037</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.01025</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.01826</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="B33" t="n">
+        <v>0.379467</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.447644</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.541805</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.598538</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.01084</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.02136</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="B34" t="n">
+        <v>0.389695</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.454245</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.559568</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.607681</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.01023</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.01776</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="B35" t="n">
+        <v>0.399326</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.459796</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.57391</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.614924</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.00963</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.01434</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="B36" t="n">
+        <v>0.408464</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.465046</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.587325</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.622903</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.009140000000000001</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.01341</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="B37" t="n">
+        <v>0.417213</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.470276</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.599646</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.630815</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.008750000000000001</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.01232</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="B38" t="n">
+        <v>0.425932</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.475831</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.61175</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.63922</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.00872</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.0121</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="B39" t="n">
+        <v>0.434422</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.48163</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.623825</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.648253</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.008489999999999999</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.01207</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="B40" t="n">
+        <v>0.442746</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.487758</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.636167</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.658107</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.008319999999999999</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.01234</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="B41" t="n">
+        <v>0.450961</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.494297</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.648895</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.668816</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.00822</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.01273</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="B42" t="n">
+        <v>0.459115</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.501328</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.662076</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.680397</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.008149999999999999</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.01318</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="B43" t="n">
+        <v>0.467458</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.509132</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.6764559999999999</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.693671</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.00834</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.01438</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="B44" t="n">
+        <v>0.475829</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.51763</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.691736</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.708368</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.008370000000000001</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.01528</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0.484269</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.526926</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.7081769999999999</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.72492</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.00844</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.01644</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="B46" t="n">
+        <v>0.492844</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.537125</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.725702</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.743511</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.008569999999999999</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.01753</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="B47" t="n">
+        <v>0.501673</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.548311</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.744897</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.765387</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.008829999999999999</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.0192</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="B48" t="n">
+        <v>0.511173</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.560768</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.765012</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.790631</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.02011</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="B49" t="n">
+        <v>0.5214569999999999</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.574567</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.785358</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.819986</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.01028</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.02035</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="B50" t="n">
+        <v>0.532753</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.590846</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.804759</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.852447</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.0113</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.0194</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="B51" t="n">
+        <v>0.5444639999999999</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.609648</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.82307</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.879233</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.01171</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.01831</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="B52" t="n">
+        <v>0.554953</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.614523</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.837167</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.888314</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.01049</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.0141</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="B53" t="n">
+        <v>0.563672</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.613865</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.847333</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.888998</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.00872</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.01017</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="B54" t="n">
+        <v>0.570932</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.612673</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.8549909999999999</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.889037</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.00726</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.00766</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="B55" t="n">
+        <v>0.577049</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.611262</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.860281</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.887954</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.00612</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.00529</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="B56" t="n">
+        <v>0.582152</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.609647</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.865878</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.888622</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.0056</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="B57" t="n">
+        <v>0.586368</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.607845</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.869839</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.888306</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.00422</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.00396</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="B58" t="n">
+        <v>0.5900339999999999</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.6061609999999999</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.873152</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.888008</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.00367</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.00331</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="B59" t="n">
+        <v>0.5931650000000001</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.604614</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.875918</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.8876810000000001</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.00313</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.00277</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="B60" t="n">
+        <v>0.5958909999999999</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.603365</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.877881</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.886921</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.00273</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.00196</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="B61" t="n">
+        <v>0.598401</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0.602426</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.880067</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.886856</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.00251</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.00219</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="B62" t="n">
+        <v>0.600665</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0.601593</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.8816659999999999</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.886451</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.00226</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.0016</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="B63" t="n">
+        <v>0.602885</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0.601001</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.883062</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.8861</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.00222</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.0014</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="B64" t="n">
+        <v>0.604772</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0.600359</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.884161</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.885675</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.00189</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.0011</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="B65" t="n">
+        <v>0.6063499999999999</v>
+      </c>
+      <c r="C65" t="n">
+        <v>0.599696</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0.884501</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.884593</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.00158</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.00034</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="B66" t="n">
+        <v>0.60756</v>
+      </c>
+      <c r="C66" t="n">
+        <v>0.598958</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0.885781</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.884827</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.00121</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.00128</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.608421</v>
+      </c>
+      <c r="C67" t="n">
+        <v>0.598167</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0.886337</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.8844070000000001</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.00086</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.00056</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.609116</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0.59751</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0.886769</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.884015</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.00043</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0.609487</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0.596819</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0.88707</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.8836310000000001</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.00037</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.0003</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.60949</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0.596055</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0.886982</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.882962</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-9.000000000000001e-05</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="B71" t="n">
+        <v>0.609158</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0.595247</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0.887074</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.882633</v>
+      </c>
+      <c r="F71" t="n">
+        <v>-0.00033</v>
+      </c>
+      <c r="G71" t="n">
+        <v>9.000000000000001e-05</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0.608502</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0.594391</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.882247</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-0.00066</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-6.999999999999999e-05</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>reflector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n_sub</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext series 550 nm</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext series Gaussian FWHM 70 nm</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>eta_ext series uniform 490-610 nm</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>EQE series 550 nm</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>EQE series Gaussian 70 nm</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.91625</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.905731</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.897125</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.242404</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.246785</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.896525</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.883149</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.873047</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.255092</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.259507</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.856164</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.845425</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.843199</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.271161</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.27448</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.782561</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.805727</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.814466</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.290872</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.291868</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.781984</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.783813</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.7877459999999999</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.310433</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.310629</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.77745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.765525</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.7541870000000001</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.330849</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.332943</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.679673</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.704476</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.71113</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.368625</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.36994</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.700986</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.699619</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.698557</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.417213</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.416427</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.710217</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.708794</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.707611</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.459115</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.45838</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.689263</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.688324</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.687566</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.501673</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.5009940000000001</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.659498</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.659123</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.658801</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.554953</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.5542049999999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.693543</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.693146</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.69282</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.586368</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.585595</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.705654</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.705299</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.705006</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.600665</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.599998</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.713441</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.7132270000000001</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.713037</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.608421</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.60786</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.713407</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.7133930000000001</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.713346</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.608502</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.6080680000000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.981425</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.976615</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.972648</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.307735</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.313344</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.9798289999999999</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.976329</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.973046</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.323594</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.330081</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.974759</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.967372</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.960599</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.344902</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.352625</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.957159</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.946866</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.94737</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.37988</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.385333</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.911254</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.928154</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.936128</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.431991</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.425178</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.931971</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.925145</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.9204560000000001</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.464183</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.464414</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.889701</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.893811</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.897822</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.520448</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.52356</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.902596</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.8996189999999999</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.8970939999999999</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.599646</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.597087</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.921121</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.919752</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.9185950000000001</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.662076</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.660733</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.917007</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.915794</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.914789</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.744897</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.743803</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.875528</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.875057</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.874654</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.837167</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.835991</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.906855</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.906388</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.906002</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.869839</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.868675</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.918532</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.9181589999999999</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.9178539999999999</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.8816659999999999</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.88056</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.923052</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.922757</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.922516</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.886337</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.88528</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.923548</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.923316</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.923125</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.885981</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Note: layer optical constants are wavelength-independent in this check, so the cut-off at n_sub = n_org = 1.8 does not move with wavelength.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2569,7 +5507,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2725,7 +5663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>